<commit_message>
Update src code for FileBrower, display AVI at 14FPS
</commit_message>
<xml_diff>
--- a/Stm32F7/STM32H723ZGT6_PIN.xlsx
+++ b/Stm32F7/STM32H723ZGT6_PIN.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\stm32_git_workspace\stm32_public_workspace\Stm32F7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5599A12A-FE85-44CF-9281-9A7D7BE09BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902B4B06-99ED-487F-928E-3AFC5C98FFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{329B8DDE-580F-4FEB-AB19-42290A552E36}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{329B8DDE-580F-4FEB-AB19-42290A552E36}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Used_Pin" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -830,50 +831,6 @@
         <a:xfrm rot="10800000">
           <a:off x="16147676" y="2207559"/>
           <a:ext cx="5572903" cy="4848902"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>578399</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>56030</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>219324</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>190499</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B52AB8E-2407-4CFC-BA80-E137139A85A9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7862223" y="2151530"/>
-          <a:ext cx="246042" cy="5658969"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2570,6 +2527,212 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25EE84AF-27ED-4850-80BA-C3133A33DA90}">
+  <dimension ref="G10:G48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="10" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G18">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G20">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G21">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G22">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G23">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G24">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G26">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G27">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G28">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G29">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G30">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G31">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G32">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G33">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G34">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G36">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G37">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G38">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G39">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G40">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G41">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="42" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G42">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G43">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G44">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G45">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="46" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G46">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="47" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G47">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G48">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74504447-645C-487A-B8A7-D9156BD79BAE}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>